<commit_message>
Finalize humanized Q2505 task and Reference
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rfc7fbf24a3e24b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R97eff2c1af5944e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -274,7 +274,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="146" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="150" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -330,7 +330,7 @@
         <x:v>原始输入文件</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>current/deployment.yaml、current/hpa.yaml、autoscaling_policy.json、environment_labels.csv和README.txt</x:v>
+        <x:v>current/deployment.yaml、current/hpa.yaml、autoscaling_policy.json和environment_labels.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -338,7 +338,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>output/release/production、output/evidence和output/README.txt</x:v>
+        <x:v>release/production/deployment.yaml、release/production/hpa.yaml、release/production/kustomization.yaml、rendered.yaml、change_record.csv和release_notes.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -346,7 +346,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>核对身份与策略→修正HPA→保护Deployment业务配置→补公共标签→组织Kustomize→kubectl构建→整理发布复核</x:v>
+        <x:v>核对身份与策略→修正HPA→保留Deployment业务配置→补公共标签→组织Kustomize→生成候选清单→记录变更</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -359,7 +359,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>指标合同</x:v>
+        <x:v>弹性指标</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
         <x:v>同时配置CPU Resource Utilization和queue_depth External AverageValue</x:v>
@@ -367,18 +367,18 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>行为合同</x:v>
+        <x:v>升降行为</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>scaleUp与scaleDown的窗口、选择规则、Percent和Pods策略逐字段取自容量合同</x:v>
+        <x:v>scaleUp与scaleDown的窗口、选择规则、Percent和Pods策略取自容量策略</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>Deployment边界</x:v>
+        <x:v>Deployment保留范围</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>metadata.labels可补公共标签，spec必须与输入Deployment完全一致</x:v>
+        <x:v>metadata.labels可以补公共标签，spec与输入Deployment保持一致</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -386,54 +386,62 @@
         <x:v>环境标签</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>production、owner和cost-center取environment_labels.csv唯一production行</x:v>
+        <x:v>production、owner和cost-center取environment_labels.csv中的production行</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>Kustomize范围</x:v>
+        <x:v>Kustomize目录</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>release/production只引用Deployment和HPA，kubectl客户端离线生成候选YAML</x:v>
+        <x:v>release/production只引用Deployment和HPA，kubectl客户端生成rendered.yaml</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>复核边界</x:v>
+        <x:v>变更记录</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>检查对象身份、HPA合同、公共标签与Deployment保护；READY只代表材料可继续审阅</x:v>
+        <x:v>change_record.csv列出HPA主要字段的前后值、来源和Deployment保留状态</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>能力边界</x:v>
+        <x:v>发布说明</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>不连接API Server，不声称HPA Controller已执行调度、指标采集或实际扩缩容</x:v>
+        <x:v>release_notes.txt说明材料用途、Deployment保留范围及客户端清单边界</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>能力边界</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>kubectl构建成功，两个对象身份正确，合同检查全部通过，Deployment.spec不变</x:v>
+        <x:v>不连接API Server，不声称HPA Controller已执行调度、指标采集或实际扩缩容</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="5" t="str">
+        <x:v>完成条件</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="str">
+        <x:v>kubectl构建成功，目标对象身份正确，HPA符合容量策略，Deployment.spec保持不变</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="5" t="str">
         <x:v>可验证点</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="str">
-        <x:v>对象复合身份、targetRef、副本边界、指标、behavior、标签、Deployment.spec和kubectl退出码</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="6" t="str">
+      <x:c r="B20" s="5" t="str">
+        <x:v>对象身份、scaleTargetRef、副本边界、metrics、behavior、公共标签、Deployment.spec和变更记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="6" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B20" s="6" t="str">
+      <x:c r="B21" s="6" t="str">
         <x:v>YAML键序、文档顺序、编辑器、临时目录、注释、排版和真实集群伸缩结果</x:v>
       </x:c>
     </x:row>

</xml_diff>